<commit_message>
Added the excel read and write changes
</commit_message>
<xml_diff>
--- a/src/test/resources/output/pro/ProExecutionData.xlsx
+++ b/src/test/resources/output/pro/ProExecutionData.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="26">
   <si>
     <t xml:space="preserve">TestCase</t>
   </si>
@@ -86,6 +86,18 @@
   </si>
   <si>
     <t>Figma</t>
+  </si>
+  <si>
+    <t>Automation Portfolio_20260910_123305_333</t>
+  </si>
+  <si>
+    <t>Automation Portfolio_20260910_134356_718</t>
+  </si>
+  <si>
+    <t>Automation Portfolio_20260910_135124_294</t>
+  </si>
+  <si>
+    <t>Automation Public Portfolio_20260910_135238_686</t>
   </si>
 </sst>
 </file>
@@ -371,11 +383,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" customWidth="true" hidden="false" style="0" width="27.15" collapsed="false" outlineLevel="0"/>
@@ -431,22 +443,22 @@
         <v>13</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C2" t="b" s="0">
         <v>0</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s" s="0">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s" s="0">
         <v>15</v>
@@ -454,16 +466,59 @@
       <c r="I2" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" t="s" s="0">
         <v>21</v>
       </c>
-      <c r="K2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" t="s">
-        <v>15</v>
-      </c>
-      <c r="M2" t="s">
+      <c r="K2" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="M2" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="0">
+        <is>
+          <t>createPublicPortfolioWithAllFields</t>
+        </is>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C3" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="J3" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="K3" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="L3" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="M3" t="s" s="0">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Deelte portfollio fix
</commit_message>
<xml_diff>
--- a/src/test/resources/output/pro/ProExecutionData.xlsx
+++ b/src/test/resources/output/pro/ProExecutionData.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="29">
   <si>
     <t xml:space="preserve">TestCase</t>
   </si>
@@ -98,6 +98,15 @@
   </si>
   <si>
     <t>Automation Public Portfolio_20260910_135238_686</t>
+  </si>
+  <si>
+    <t>Automation Portfolio_20260910_145432_471</t>
+  </si>
+  <si>
+    <t>Automation Portfolio_20260910_180809_740</t>
+  </si>
+  <si>
+    <t>Automation Public Portfolio_20260910_180946_775</t>
   </si>
 </sst>
 </file>
@@ -443,7 +452,7 @@
         <v>13</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C2" t="b" s="0">
         <v>0</v>
@@ -486,7 +495,7 @@
         </is>
       </c>
       <c r="B3" t="s" s="0">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C3" t="b" s="0">
         <v>1</v>

</xml_diff>